<commit_message>
att pedido 018 fertilidade
</commit_message>
<xml_diff>
--- a/pedidos/F2026018S.xlsx
+++ b/pedidos/F2026018S.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/icaro_ramiro_agrorobotica_com_br/Documents/Documentos/7ATVOS/7Selecao_Amostras/SAIDAS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/pedidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_C85283E02F4B4313336C5088C52A1B01197904DF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFF181A6-CFAE-4BFA-919F-FF628E9EEF78}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_C85283E02F4B4313336C5088C52A1B01197904DF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76DBB4A4-9810-4B0B-9DB0-23168C502B23}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1627" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1625" uniqueCount="259">
   <si>
     <t>Obj-ID</t>
   </si>
@@ -419,9 +419,6 @@
   </si>
   <si>
     <t>120052</t>
-  </si>
-  <si>
-    <t>UCP0480</t>
   </si>
   <si>
     <t>120091</t>
@@ -1470,31 +1467,31 @@
         <v>1</v>
       </c>
       <c r="V2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W2" t="s">
+        <v>139</v>
+      </c>
+      <c r="X2" t="s">
         <v>140</v>
       </c>
-      <c r="X2" t="s">
-        <v>141</v>
-      </c>
       <c r="Y2">
         <v>1</v>
       </c>
       <c r="AC2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:61" x14ac:dyDescent="0.25">
@@ -1550,31 +1547,31 @@
         <v>2</v>
       </c>
       <c r="V3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Y3">
         <v>2</v>
       </c>
       <c r="AC3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:61" x14ac:dyDescent="0.25">
@@ -1627,31 +1624,31 @@
         <v>1</v>
       </c>
       <c r="V4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Y4">
         <v>3</v>
       </c>
       <c r="AC4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" spans="1:61" x14ac:dyDescent="0.25">
@@ -1704,31 +1701,31 @@
         <v>2</v>
       </c>
       <c r="V5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="Y5">
         <v>4</v>
       </c>
       <c r="AC5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" spans="1:61" x14ac:dyDescent="0.25">
@@ -1784,31 +1781,31 @@
         <v>1</v>
       </c>
       <c r="V6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Y6">
         <v>5</v>
       </c>
       <c r="AC6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7" spans="1:61" x14ac:dyDescent="0.25">
@@ -1864,31 +1861,31 @@
         <v>2</v>
       </c>
       <c r="V7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="Y7">
         <v>6</v>
       </c>
       <c r="AC7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8" spans="1:61" x14ac:dyDescent="0.25">
@@ -1944,31 +1941,31 @@
         <v>1</v>
       </c>
       <c r="V8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="Y8">
         <v>7</v>
       </c>
       <c r="AC8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" spans="1:61" x14ac:dyDescent="0.25">
@@ -2024,28 +2021,28 @@
         <v>2</v>
       </c>
       <c r="V9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Y9">
         <v>8</v>
       </c>
       <c r="AC9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" spans="1:61" x14ac:dyDescent="0.25">
@@ -2101,28 +2098,28 @@
         <v>1</v>
       </c>
       <c r="V10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="Y10">
         <v>9</v>
       </c>
       <c r="AC10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:61" x14ac:dyDescent="0.25">
@@ -2178,28 +2175,28 @@
         <v>2</v>
       </c>
       <c r="V11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="Y11">
         <v>10</v>
       </c>
       <c r="AC11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" spans="1:61" x14ac:dyDescent="0.25">
@@ -2255,28 +2252,28 @@
         <v>1</v>
       </c>
       <c r="V12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Y12">
         <v>11</v>
       </c>
       <c r="AC12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:61" x14ac:dyDescent="0.25">
@@ -2332,28 +2329,28 @@
         <v>2</v>
       </c>
       <c r="V13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Y13">
         <v>12</v>
       </c>
       <c r="AC13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" spans="1:61" x14ac:dyDescent="0.25">
@@ -2409,28 +2406,28 @@
         <v>1</v>
       </c>
       <c r="V14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="Y14">
         <v>13</v>
       </c>
       <c r="AC14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" spans="1:61" x14ac:dyDescent="0.25">
@@ -2486,28 +2483,28 @@
         <v>2</v>
       </c>
       <c r="V15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="Y15">
         <v>14</v>
       </c>
       <c r="AC15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" spans="1:61" x14ac:dyDescent="0.25">
@@ -2563,28 +2560,28 @@
         <v>1</v>
       </c>
       <c r="V16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Y16">
         <v>15</v>
       </c>
       <c r="AC16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.25">
@@ -2640,28 +2637,28 @@
         <v>2</v>
       </c>
       <c r="V17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Y17">
         <v>16</v>
       </c>
       <c r="AC17" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF17" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH17" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI17" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="18" spans="1:35" x14ac:dyDescent="0.25">
@@ -2714,28 +2711,28 @@
         <v>1</v>
       </c>
       <c r="V18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W18" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Y18">
         <v>17</v>
       </c>
       <c r="AC18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="19" spans="1:35" x14ac:dyDescent="0.25">
@@ -2788,28 +2785,28 @@
         <v>2</v>
       </c>
       <c r="V19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="Y19">
         <v>18</v>
       </c>
       <c r="AC19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="20" spans="1:35" x14ac:dyDescent="0.25">
@@ -2865,31 +2862,31 @@
         <v>1</v>
       </c>
       <c r="V20" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="Y20">
         <v>19</v>
       </c>
       <c r="AC20" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE20" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF20" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH20" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI20" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="21" spans="1:35" x14ac:dyDescent="0.25">
@@ -2945,31 +2942,31 @@
         <v>2</v>
       </c>
       <c r="V21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W21" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X21" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Y21">
         <v>20</v>
       </c>
       <c r="AC21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="22" spans="1:35" x14ac:dyDescent="0.25">
@@ -3025,31 +3022,31 @@
         <v>1</v>
       </c>
       <c r="V22" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W22" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X22" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Y22">
         <v>21</v>
       </c>
       <c r="AC22" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE22" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF22" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH22" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI22" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23" spans="1:35" x14ac:dyDescent="0.25">
@@ -3105,28 +3102,28 @@
         <v>2</v>
       </c>
       <c r="V23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Y23">
         <v>22</v>
       </c>
       <c r="AC23" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF23" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH23" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI23" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="24" spans="1:35" x14ac:dyDescent="0.25">
@@ -3182,28 +3179,28 @@
         <v>1</v>
       </c>
       <c r="V24" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X24" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Y24">
         <v>23</v>
       </c>
       <c r="AC24" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF24" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH24" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI24" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="25" spans="1:35" x14ac:dyDescent="0.25">
@@ -3259,28 +3256,28 @@
         <v>2</v>
       </c>
       <c r="V25" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W25" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X25" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Y25">
         <v>24</v>
       </c>
       <c r="AC25" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF25" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH25" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI25" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26" spans="1:35" x14ac:dyDescent="0.25">
@@ -3336,28 +3333,28 @@
         <v>1</v>
       </c>
       <c r="V26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X26" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Y26">
         <v>25</v>
       </c>
       <c r="AC26" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF26" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH26" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI26" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="27" spans="1:35" x14ac:dyDescent="0.25">
@@ -3413,28 +3410,28 @@
         <v>2</v>
       </c>
       <c r="V27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W27" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="Y27">
         <v>26</v>
       </c>
       <c r="AC27" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF27" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH27" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI27" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="28" spans="1:35" x14ac:dyDescent="0.25">
@@ -3490,31 +3487,31 @@
         <v>1</v>
       </c>
       <c r="V28" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W28" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Y28">
         <v>27</v>
       </c>
       <c r="AC28" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE28" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF28" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH28" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI28" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="29" spans="1:35" x14ac:dyDescent="0.25">
@@ -3570,31 +3567,31 @@
         <v>2</v>
       </c>
       <c r="V29" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Y29">
         <v>28</v>
       </c>
       <c r="AC29" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE29" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF29" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH29" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI29" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="30" spans="1:35" x14ac:dyDescent="0.25">
@@ -3650,31 +3647,31 @@
         <v>1</v>
       </c>
       <c r="V30" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W30" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X30" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Y30">
         <v>29</v>
       </c>
       <c r="AC30" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE30" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF30" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH30" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI30" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="31" spans="1:35" x14ac:dyDescent="0.25">
@@ -3730,28 +3727,28 @@
         <v>2</v>
       </c>
       <c r="V31" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X31" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Y31">
         <v>30</v>
       </c>
       <c r="AC31" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF31" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH31" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI31" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="32" spans="1:35" x14ac:dyDescent="0.25">
@@ -3807,28 +3804,28 @@
         <v>1</v>
       </c>
       <c r="V32" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W32" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X32" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Y32">
         <v>31</v>
       </c>
       <c r="AC32" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF32" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH32" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI32" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="33" spans="1:35" x14ac:dyDescent="0.25">
@@ -3884,28 +3881,28 @@
         <v>2</v>
       </c>
       <c r="V33" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W33" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X33" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Y33">
         <v>32</v>
       </c>
       <c r="AC33" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF33" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH33" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI33" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="34" spans="1:35" x14ac:dyDescent="0.25">
@@ -3961,28 +3958,28 @@
         <v>1</v>
       </c>
       <c r="V34" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W34" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="Y34">
         <v>33</v>
       </c>
       <c r="AC34" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF34" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH34" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI34" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="35" spans="1:35" x14ac:dyDescent="0.25">
@@ -4038,28 +4035,28 @@
         <v>2</v>
       </c>
       <c r="V35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W35" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X35" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Y35">
         <v>34</v>
       </c>
       <c r="AC35" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF35" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH35" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI35" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="36" spans="1:35" x14ac:dyDescent="0.25">
@@ -4115,28 +4112,28 @@
         <v>1</v>
       </c>
       <c r="V36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X36" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="Y36">
         <v>35</v>
       </c>
       <c r="AC36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="37" spans="1:35" x14ac:dyDescent="0.25">
@@ -4192,28 +4189,28 @@
         <v>2</v>
       </c>
       <c r="V37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W37" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Y37">
         <v>36</v>
       </c>
       <c r="AC37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="38" spans="1:35" x14ac:dyDescent="0.25">
@@ -4269,28 +4266,28 @@
         <v>1</v>
       </c>
       <c r="V38" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Y38">
         <v>37</v>
       </c>
       <c r="AC38" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF38" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH38" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI38" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="39" spans="1:35" x14ac:dyDescent="0.25">
@@ -4346,28 +4343,28 @@
         <v>2</v>
       </c>
       <c r="V39" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W39" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X39" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Y39">
         <v>38</v>
       </c>
       <c r="AC39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="40" spans="1:35" x14ac:dyDescent="0.25">
@@ -4423,28 +4420,28 @@
         <v>1</v>
       </c>
       <c r="V40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W40" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Y40">
         <v>39</v>
       </c>
       <c r="AC40" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF40" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH40" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI40" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" spans="1:35" x14ac:dyDescent="0.25">
@@ -4500,28 +4497,28 @@
         <v>2</v>
       </c>
       <c r="V41" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W41" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X41" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="Y41">
         <v>40</v>
       </c>
       <c r="AC41" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF41" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH41" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI41" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:35" x14ac:dyDescent="0.25">
@@ -4577,28 +4574,28 @@
         <v>1</v>
       </c>
       <c r="V42" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W42" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X42" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Y42">
         <v>41</v>
       </c>
       <c r="AC42" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF42" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH42" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI42" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="43" spans="1:35" x14ac:dyDescent="0.25">
@@ -4654,28 +4651,28 @@
         <v>2</v>
       </c>
       <c r="V43" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W43" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X43" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Y43">
         <v>42</v>
       </c>
       <c r="AC43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="44" spans="1:35" x14ac:dyDescent="0.25">
@@ -4731,28 +4728,28 @@
         <v>1</v>
       </c>
       <c r="V44" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W44" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X44" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Y44">
         <v>43</v>
       </c>
       <c r="AC44" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF44" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH44" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI44" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="45" spans="1:35" x14ac:dyDescent="0.25">
@@ -4808,28 +4805,28 @@
         <v>2</v>
       </c>
       <c r="V45" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W45" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Y45">
         <v>44</v>
       </c>
       <c r="AC45" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF45" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH45" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI45" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="46" spans="1:35" x14ac:dyDescent="0.25">
@@ -4885,31 +4882,31 @@
         <v>1</v>
       </c>
       <c r="V46" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W46" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X46" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y46">
         <v>45</v>
       </c>
       <c r="AC46" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE46" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF46" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH46" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI46" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="47" spans="1:35" x14ac:dyDescent="0.25">
@@ -4965,31 +4962,31 @@
         <v>2</v>
       </c>
       <c r="V47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W47" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X47" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Y47">
         <v>46</v>
       </c>
       <c r="AC47" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE47" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF47" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH47" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI47" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="48" spans="1:35" x14ac:dyDescent="0.25">
@@ -5045,31 +5042,31 @@
         <v>1</v>
       </c>
       <c r="V48" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W48" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X48" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Y48">
         <v>47</v>
       </c>
       <c r="AC48" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE48" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF48" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH48" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI48" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="49" spans="1:35" x14ac:dyDescent="0.25">
@@ -5125,28 +5122,28 @@
         <v>2</v>
       </c>
       <c r="V49" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W49" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X49" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Y49">
         <v>48</v>
       </c>
       <c r="AC49" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF49" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH49" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI49" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="50" spans="1:35" x14ac:dyDescent="0.25">
@@ -5202,28 +5199,28 @@
         <v>1</v>
       </c>
       <c r="V50" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W50" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X50" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="Y50">
         <v>49</v>
       </c>
       <c r="AC50" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF50" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH50" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI50" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="51" spans="1:35" x14ac:dyDescent="0.25">
@@ -5279,28 +5276,28 @@
         <v>2</v>
       </c>
       <c r="V51" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W51" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X51" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Y51">
         <v>50</v>
       </c>
       <c r="AC51" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF51" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH51" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI51" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="52" spans="1:35" x14ac:dyDescent="0.25">
@@ -5356,28 +5353,28 @@
         <v>1</v>
       </c>
       <c r="V52" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W52" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X52" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Y52">
         <v>51</v>
       </c>
       <c r="AC52" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF52" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH52" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI52" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="53" spans="1:35" x14ac:dyDescent="0.25">
@@ -5433,28 +5430,28 @@
         <v>2</v>
       </c>
       <c r="V53" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W53" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X53" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="Y53">
         <v>52</v>
       </c>
       <c r="AC53" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF53" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH53" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI53" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="54" spans="1:35" x14ac:dyDescent="0.25">
@@ -5510,28 +5507,28 @@
         <v>1</v>
       </c>
       <c r="V54" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W54" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X54" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Y54">
         <v>53</v>
       </c>
       <c r="AC54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="55" spans="1:35" x14ac:dyDescent="0.25">
@@ -5587,28 +5584,28 @@
         <v>2</v>
       </c>
       <c r="V55" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W55" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X55" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="Y55">
         <v>54</v>
       </c>
       <c r="AC55" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF55" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH55" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI55" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="56" spans="1:35" x14ac:dyDescent="0.25">
@@ -5664,28 +5661,28 @@
         <v>1</v>
       </c>
       <c r="V56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W56" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X56" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="Y56">
         <v>55</v>
       </c>
       <c r="AC56" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF56" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH56" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI56" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="57" spans="1:35" x14ac:dyDescent="0.25">
@@ -5741,28 +5738,28 @@
         <v>2</v>
       </c>
       <c r="V57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W57" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X57" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Y57">
         <v>56</v>
       </c>
       <c r="AC57" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF57" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH57" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI57" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="58" spans="1:35" x14ac:dyDescent="0.25">
@@ -5818,28 +5815,28 @@
         <v>1</v>
       </c>
       <c r="V58" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W58" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X58" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Y58">
         <v>57</v>
       </c>
       <c r="AC58" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF58" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH58" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI58" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="59" spans="1:35" x14ac:dyDescent="0.25">
@@ -5895,28 +5892,28 @@
         <v>2</v>
       </c>
       <c r="V59" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W59" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X59" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="Y59">
         <v>58</v>
       </c>
       <c r="AC59" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF59" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH59" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI59" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="60" spans="1:35" x14ac:dyDescent="0.25">
@@ -5972,31 +5969,31 @@
         <v>1</v>
       </c>
       <c r="V60" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W60" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X60" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Y60">
         <v>59</v>
       </c>
       <c r="AC60" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE60" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF60" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH60" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI60" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="61" spans="1:35" x14ac:dyDescent="0.25">
@@ -6052,31 +6049,31 @@
         <v>2</v>
       </c>
       <c r="V61" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W61" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X61" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Y61">
         <v>60</v>
       </c>
       <c r="AC61" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE61" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF61" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH61" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI61" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="62" spans="1:35" x14ac:dyDescent="0.25">
@@ -6132,28 +6129,28 @@
         <v>1</v>
       </c>
       <c r="V62" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W62" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X62" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Y62">
         <v>61</v>
       </c>
       <c r="AC62" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF62" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH62" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI62" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="63" spans="1:35" x14ac:dyDescent="0.25">
@@ -6209,28 +6206,28 @@
         <v>2</v>
       </c>
       <c r="V63" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W63" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X63" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Y63">
         <v>62</v>
       </c>
       <c r="AC63" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF63" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH63" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI63" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="64" spans="1:35" x14ac:dyDescent="0.25">
@@ -6286,31 +6283,31 @@
         <v>1</v>
       </c>
       <c r="V64" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W64" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X64" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Y64">
         <v>63</v>
       </c>
       <c r="AC64" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE64" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF64" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH64" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI64" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="65" spans="1:35" x14ac:dyDescent="0.25">
@@ -6366,31 +6363,31 @@
         <v>2</v>
       </c>
       <c r="V65" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W65" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X65" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="Y65">
         <v>64</v>
       </c>
       <c r="AC65" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE65" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF65" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH65" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI65" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="66" spans="1:35" x14ac:dyDescent="0.25">
@@ -6446,31 +6443,31 @@
         <v>1</v>
       </c>
       <c r="V66" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W66" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X66" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Y66">
         <v>65</v>
       </c>
       <c r="AC66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="67" spans="1:35" x14ac:dyDescent="0.25">
@@ -6526,31 +6523,31 @@
         <v>2</v>
       </c>
       <c r="V67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W67" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X67" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y67">
         <v>66</v>
       </c>
       <c r="AC67" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE67" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF67" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH67" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI67" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="68" spans="1:35" x14ac:dyDescent="0.25">
@@ -6606,31 +6603,31 @@
         <v>1</v>
       </c>
       <c r="V68" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W68" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X68" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Y68">
         <v>67</v>
       </c>
       <c r="AC68" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE68" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF68" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH68" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI68" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="69" spans="1:35" x14ac:dyDescent="0.25">
@@ -6686,28 +6683,28 @@
         <v>2</v>
       </c>
       <c r="V69" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W69" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X69" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Y69">
         <v>68</v>
       </c>
       <c r="AC69" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF69" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH69" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI69" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="70" spans="1:35" x14ac:dyDescent="0.25">
@@ -6763,28 +6760,28 @@
         <v>1</v>
       </c>
       <c r="V70" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W70" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X70" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Y70">
         <v>69</v>
       </c>
       <c r="AC70" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF70" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH70" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI70" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="71" spans="1:35" x14ac:dyDescent="0.25">
@@ -6840,28 +6837,28 @@
         <v>2</v>
       </c>
       <c r="V71" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W71" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X71" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="Y71">
         <v>70</v>
       </c>
       <c r="AC71" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF71" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH71" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI71" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="72" spans="1:35" x14ac:dyDescent="0.25">
@@ -6917,28 +6914,28 @@
         <v>1</v>
       </c>
       <c r="V72" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W72" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X72" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="Y72">
         <v>71</v>
       </c>
       <c r="AC72" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF72" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH72" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI72" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="73" spans="1:35" x14ac:dyDescent="0.25">
@@ -6994,28 +6991,28 @@
         <v>2</v>
       </c>
       <c r="V73" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W73" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X73" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Y73">
         <v>72</v>
       </c>
       <c r="AC73" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF73" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH73" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI73" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="74" spans="1:35" x14ac:dyDescent="0.25">
@@ -7071,28 +7068,28 @@
         <v>1</v>
       </c>
       <c r="V74" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W74" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X74" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Y74">
         <v>73</v>
       </c>
       <c r="AC74" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF74" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH74" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI74" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="75" spans="1:35" x14ac:dyDescent="0.25">
@@ -7148,28 +7145,28 @@
         <v>2</v>
       </c>
       <c r="V75" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W75" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X75" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="Y75">
         <v>74</v>
       </c>
       <c r="AC75" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF75" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH75" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI75" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="76" spans="1:35" x14ac:dyDescent="0.25">
@@ -7225,28 +7222,28 @@
         <v>1</v>
       </c>
       <c r="V76" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W76" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X76" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="Y76">
         <v>75</v>
       </c>
       <c r="AC76" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF76" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH76" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI76" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="77" spans="1:35" x14ac:dyDescent="0.25">
@@ -7302,28 +7299,28 @@
         <v>2</v>
       </c>
       <c r="V77" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W77" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X77" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Y77">
         <v>76</v>
       </c>
       <c r="AC77" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF77" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH77" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI77" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="78" spans="1:35" x14ac:dyDescent="0.25">
@@ -7379,28 +7376,28 @@
         <v>1</v>
       </c>
       <c r="V78" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W78" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X78" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="Y78">
         <v>77</v>
       </c>
       <c r="AC78" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF78" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH78" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI78" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="79" spans="1:35" x14ac:dyDescent="0.25">
@@ -7456,28 +7453,28 @@
         <v>2</v>
       </c>
       <c r="V79" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W79" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X79" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="Y79">
         <v>78</v>
       </c>
       <c r="AC79" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF79" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH79" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI79" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="80" spans="1:35" x14ac:dyDescent="0.25">
@@ -7533,28 +7530,28 @@
         <v>1</v>
       </c>
       <c r="V80" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W80" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X80" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Y80">
         <v>79</v>
       </c>
       <c r="AC80" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF80" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH80" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI80" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="81" spans="1:35" x14ac:dyDescent="0.25">
@@ -7610,28 +7607,28 @@
         <v>2</v>
       </c>
       <c r="V81" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W81" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X81" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="Y81">
         <v>80</v>
       </c>
       <c r="AC81" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF81" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH81" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI81" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="82" spans="1:35" x14ac:dyDescent="0.25">
@@ -7687,28 +7684,28 @@
         <v>1</v>
       </c>
       <c r="V82" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W82" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X82" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="Y82">
         <v>81</v>
       </c>
       <c r="AC82" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF82" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH82" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI82" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="83" spans="1:35" x14ac:dyDescent="0.25">
@@ -7764,28 +7761,28 @@
         <v>2</v>
       </c>
       <c r="V83" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W83" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X83" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Y83">
         <v>82</v>
       </c>
       <c r="AC83" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF83" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH83" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI83" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="84" spans="1:35" x14ac:dyDescent="0.25">
@@ -7841,31 +7838,31 @@
         <v>1</v>
       </c>
       <c r="V84" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W84" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X84" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Y84">
         <v>83</v>
       </c>
       <c r="AC84" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE84" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF84" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH84" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI84" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="85" spans="1:35" x14ac:dyDescent="0.25">
@@ -7921,28 +7918,28 @@
         <v>2</v>
       </c>
       <c r="V85" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W85" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X85" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Y85">
         <v>84</v>
       </c>
       <c r="AC85" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF85" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH85" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI85" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="86" spans="1:35" x14ac:dyDescent="0.25">
@@ -7998,28 +7995,28 @@
         <v>1</v>
       </c>
       <c r="V86" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W86" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X86" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="Y86">
         <v>85</v>
       </c>
       <c r="AC86" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF86" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH86" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI86" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="87" spans="1:35" x14ac:dyDescent="0.25">
@@ -8075,28 +8072,28 @@
         <v>2</v>
       </c>
       <c r="V87" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W87" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X87" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="Y87">
         <v>86</v>
       </c>
       <c r="AC87" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF87" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH87" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI87" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="88" spans="1:35" x14ac:dyDescent="0.25">
@@ -8136,8 +8133,8 @@
       <c r="M88" t="s">
         <v>123</v>
       </c>
-      <c r="O88" t="s">
-        <v>133</v>
+      <c r="O88">
+        <v>120480</v>
       </c>
       <c r="P88">
         <v>1</v>
@@ -8152,31 +8149,31 @@
         <v>1</v>
       </c>
       <c r="V88" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W88" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X88" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="Y88">
         <v>87</v>
       </c>
       <c r="AC88" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE88" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF88" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH88" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI88" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="89" spans="1:35" x14ac:dyDescent="0.25">
@@ -8216,8 +8213,8 @@
       <c r="M89" t="s">
         <v>123</v>
       </c>
-      <c r="O89" t="s">
-        <v>133</v>
+      <c r="O89">
+        <v>120480</v>
       </c>
       <c r="P89">
         <v>1</v>
@@ -8232,31 +8229,31 @@
         <v>2</v>
       </c>
       <c r="V89" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W89" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X89" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="Y89">
         <v>88</v>
       </c>
       <c r="AC89" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE89" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF89" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH89" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI89" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="90" spans="1:35" x14ac:dyDescent="0.25">
@@ -8297,7 +8294,7 @@
         <v>123</v>
       </c>
       <c r="O90" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P90">
         <v>1</v>
@@ -8312,31 +8309,31 @@
         <v>1</v>
       </c>
       <c r="V90" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W90" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X90" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="Y90">
         <v>89</v>
       </c>
       <c r="AC90" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE90" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF90" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH90" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI90" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="91" spans="1:35" x14ac:dyDescent="0.25">
@@ -8377,7 +8374,7 @@
         <v>123</v>
       </c>
       <c r="O91" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P91">
         <v>1</v>
@@ -8392,31 +8389,31 @@
         <v>2</v>
       </c>
       <c r="V91" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W91" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="Y91">
         <v>90</v>
       </c>
       <c r="AC91" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE91" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF91" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH91" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI91" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="92" spans="1:35" x14ac:dyDescent="0.25">
@@ -8457,7 +8454,7 @@
         <v>123</v>
       </c>
       <c r="O92" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P92">
         <v>1</v>
@@ -8472,31 +8469,31 @@
         <v>1</v>
       </c>
       <c r="V92" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W92" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X92" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="Y92">
         <v>91</v>
       </c>
       <c r="AC92" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE92" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF92" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH92" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI92" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="93" spans="1:35" x14ac:dyDescent="0.25">
@@ -8537,7 +8534,7 @@
         <v>123</v>
       </c>
       <c r="O93" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P93">
         <v>1</v>
@@ -8552,31 +8549,31 @@
         <v>2</v>
       </c>
       <c r="V93" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X93" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="Y93">
         <v>92</v>
       </c>
       <c r="AC93" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE93" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF93" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH93" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI93" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="94" spans="1:35" x14ac:dyDescent="0.25">
@@ -8617,7 +8614,7 @@
         <v>123</v>
       </c>
       <c r="O94" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P94">
         <v>1</v>
@@ -8632,28 +8629,28 @@
         <v>1</v>
       </c>
       <c r="V94" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W94" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X94" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="Y94">
         <v>93</v>
       </c>
       <c r="AC94" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF94" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH94" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI94" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="95" spans="1:35" x14ac:dyDescent="0.25">
@@ -8694,7 +8691,7 @@
         <v>123</v>
       </c>
       <c r="O95" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P95">
         <v>1</v>
@@ -8709,28 +8706,28 @@
         <v>2</v>
       </c>
       <c r="V95" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W95" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X95" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="Y95">
         <v>94</v>
       </c>
       <c r="AC95" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF95" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH95" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI95" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="96" spans="1:35" x14ac:dyDescent="0.25">
@@ -8771,7 +8768,7 @@
         <v>123</v>
       </c>
       <c r="O96" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P96">
         <v>1</v>
@@ -8786,31 +8783,31 @@
         <v>1</v>
       </c>
       <c r="V96" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W96" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X96" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="Y96">
         <v>95</v>
       </c>
       <c r="AC96" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE96" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF96" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH96" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI96" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="97" spans="1:35" x14ac:dyDescent="0.25">
@@ -8851,7 +8848,7 @@
         <v>123</v>
       </c>
       <c r="O97" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P97">
         <v>1</v>
@@ -8866,31 +8863,31 @@
         <v>2</v>
       </c>
       <c r="V97" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W97" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X97" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Y97">
         <v>96</v>
       </c>
       <c r="AC97" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE97" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF97" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH97" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI97" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="98" spans="1:35" x14ac:dyDescent="0.25">
@@ -8931,7 +8928,7 @@
         <v>123</v>
       </c>
       <c r="O98" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P98">
         <v>1</v>
@@ -8946,31 +8943,31 @@
         <v>1</v>
       </c>
       <c r="V98" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W98" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X98" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="Y98">
         <v>97</v>
       </c>
       <c r="AC98" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE98" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF98" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH98" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI98" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="99" spans="1:35" x14ac:dyDescent="0.25">
@@ -9011,7 +9008,7 @@
         <v>123</v>
       </c>
       <c r="O99" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P99">
         <v>1</v>
@@ -9026,28 +9023,28 @@
         <v>2</v>
       </c>
       <c r="V99" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W99" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X99" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Y99">
         <v>98</v>
       </c>
       <c r="AC99" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF99" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH99" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI99" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="100" spans="1:35" x14ac:dyDescent="0.25">
@@ -9088,7 +9085,7 @@
         <v>123</v>
       </c>
       <c r="O100" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P100">
         <v>1</v>
@@ -9103,28 +9100,28 @@
         <v>1</v>
       </c>
       <c r="V100" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W100" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X100" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="Y100">
         <v>99</v>
       </c>
       <c r="AC100" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF100" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH100" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI100" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="101" spans="1:35" x14ac:dyDescent="0.25">
@@ -9165,7 +9162,7 @@
         <v>123</v>
       </c>
       <c r="O101" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P101">
         <v>1</v>
@@ -9180,28 +9177,28 @@
         <v>2</v>
       </c>
       <c r="V101" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W101" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X101" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Y101">
         <v>100</v>
       </c>
       <c r="AC101" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF101" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH101" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI101" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="102" spans="1:35" x14ac:dyDescent="0.25">
@@ -9242,7 +9239,7 @@
         <v>123</v>
       </c>
       <c r="O102" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P102">
         <v>1</v>
@@ -9257,28 +9254,28 @@
         <v>1</v>
       </c>
       <c r="V102" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W102" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X102" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="Y102">
         <v>101</v>
       </c>
       <c r="AC102" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF102" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH102" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI102" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="103" spans="1:35" x14ac:dyDescent="0.25">
@@ -9319,7 +9316,7 @@
         <v>123</v>
       </c>
       <c r="O103" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P103">
         <v>1</v>
@@ -9334,28 +9331,28 @@
         <v>2</v>
       </c>
       <c r="V103" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W103" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X103" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="Y103">
         <v>102</v>
       </c>
       <c r="AC103" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF103" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH103" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI103" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="104" spans="1:35" x14ac:dyDescent="0.25">
@@ -9396,7 +9393,7 @@
         <v>123</v>
       </c>
       <c r="O104" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P104">
         <v>1</v>
@@ -9411,28 +9408,28 @@
         <v>1</v>
       </c>
       <c r="V104" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W104" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X104" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="Y104">
         <v>103</v>
       </c>
       <c r="AC104" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF104" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH104" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI104" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="105" spans="1:35" x14ac:dyDescent="0.25">
@@ -9473,7 +9470,7 @@
         <v>123</v>
       </c>
       <c r="O105" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P105">
         <v>1</v>
@@ -9488,28 +9485,28 @@
         <v>2</v>
       </c>
       <c r="V105" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W105" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X105" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y105">
         <v>104</v>
       </c>
       <c r="AC105" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF105" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH105" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI105" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="106" spans="1:35" x14ac:dyDescent="0.25">
@@ -9550,7 +9547,7 @@
         <v>123</v>
       </c>
       <c r="O106" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P106">
         <v>1</v>
@@ -9565,28 +9562,28 @@
         <v>1</v>
       </c>
       <c r="V106" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W106" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X106" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="Y106">
         <v>105</v>
       </c>
       <c r="AC106" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF106" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH106" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI106" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="107" spans="1:35" x14ac:dyDescent="0.25">
@@ -9627,7 +9624,7 @@
         <v>123</v>
       </c>
       <c r="O107" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P107">
         <v>1</v>
@@ -9642,28 +9639,28 @@
         <v>2</v>
       </c>
       <c r="V107" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W107" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X107" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="Y107">
         <v>106</v>
       </c>
       <c r="AC107" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF107" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH107" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI107" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="108" spans="1:35" x14ac:dyDescent="0.25">
@@ -9704,7 +9701,7 @@
         <v>123</v>
       </c>
       <c r="O108" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P108">
         <v>1</v>
@@ -9719,31 +9716,31 @@
         <v>1</v>
       </c>
       <c r="V108" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W108" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X108" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="Y108">
         <v>107</v>
       </c>
       <c r="AC108" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE108" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF108" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH108" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI108" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="109" spans="1:35" x14ac:dyDescent="0.25">
@@ -9784,7 +9781,7 @@
         <v>123</v>
       </c>
       <c r="O109" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P109">
         <v>1</v>
@@ -9799,31 +9796,31 @@
         <v>2</v>
       </c>
       <c r="V109" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W109" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X109" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="Y109">
         <v>108</v>
       </c>
       <c r="AC109" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE109" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF109" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH109" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI109" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="110" spans="1:35" x14ac:dyDescent="0.25">
@@ -9864,7 +9861,7 @@
         <v>123</v>
       </c>
       <c r="O110" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P110">
         <v>1</v>
@@ -9879,31 +9876,31 @@
         <v>1</v>
       </c>
       <c r="V110" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W110" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X110" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="Y110">
         <v>109</v>
       </c>
       <c r="AC110" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AE110" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF110" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH110" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI110" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="111" spans="1:35" x14ac:dyDescent="0.25">
@@ -9944,7 +9941,7 @@
         <v>123</v>
       </c>
       <c r="O111" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P111">
         <v>1</v>
@@ -9959,28 +9956,28 @@
         <v>2</v>
       </c>
       <c r="V111" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W111" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X111" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Y111">
         <v>110</v>
       </c>
       <c r="AC111" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF111" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH111" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI111" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="112" spans="1:35" x14ac:dyDescent="0.25">
@@ -10021,7 +10018,7 @@
         <v>123</v>
       </c>
       <c r="O112" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P112">
         <v>1</v>
@@ -10036,28 +10033,28 @@
         <v>1</v>
       </c>
       <c r="V112" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W112" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X112" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="Y112">
         <v>111</v>
       </c>
       <c r="AC112" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF112" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH112" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI112" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="113" spans="1:35" x14ac:dyDescent="0.25">
@@ -10098,7 +10095,7 @@
         <v>123</v>
       </c>
       <c r="O113" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P113">
         <v>1</v>
@@ -10113,28 +10110,28 @@
         <v>2</v>
       </c>
       <c r="V113" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W113" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X113" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="Y113">
         <v>112</v>
       </c>
       <c r="AC113" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF113" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH113" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI113" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="114" spans="1:35" x14ac:dyDescent="0.25">
@@ -10175,7 +10172,7 @@
         <v>123</v>
       </c>
       <c r="O114" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P114">
         <v>1</v>
@@ -10190,28 +10187,28 @@
         <v>1</v>
       </c>
       <c r="V114" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W114" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X114" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="Y114">
         <v>113</v>
       </c>
       <c r="AC114" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF114" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH114" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI114" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="115" spans="1:35" x14ac:dyDescent="0.25">
@@ -10252,7 +10249,7 @@
         <v>123</v>
       </c>
       <c r="O115" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P115">
         <v>1</v>
@@ -10267,28 +10264,28 @@
         <v>2</v>
       </c>
       <c r="V115" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W115" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X115" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="Y115">
         <v>114</v>
       </c>
       <c r="AC115" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF115" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH115" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI115" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="116" spans="1:35" x14ac:dyDescent="0.25">
@@ -10329,7 +10326,7 @@
         <v>123</v>
       </c>
       <c r="O116" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P116">
         <v>1</v>
@@ -10344,28 +10341,28 @@
         <v>1</v>
       </c>
       <c r="V116" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W116" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X116" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="Y116">
         <v>115</v>
       </c>
       <c r="AC116" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF116" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH116" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI116" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="117" spans="1:35" x14ac:dyDescent="0.25">
@@ -10406,7 +10403,7 @@
         <v>123</v>
       </c>
       <c r="O117" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P117">
         <v>1</v>
@@ -10421,28 +10418,28 @@
         <v>2</v>
       </c>
       <c r="V117" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W117" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X117" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Y117">
         <v>116</v>
       </c>
       <c r="AC117" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF117" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH117" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI117" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="118" spans="1:35" x14ac:dyDescent="0.25">
@@ -10483,7 +10480,7 @@
         <v>123</v>
       </c>
       <c r="O118" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P118">
         <v>1</v>
@@ -10498,28 +10495,28 @@
         <v>1</v>
       </c>
       <c r="V118" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W118" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X118" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="Y118">
         <v>117</v>
       </c>
       <c r="AC118" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF118" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH118" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI118" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="119" spans="1:35" x14ac:dyDescent="0.25">
@@ -10560,7 +10557,7 @@
         <v>123</v>
       </c>
       <c r="O119" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P119">
         <v>1</v>
@@ -10575,28 +10572,28 @@
         <v>2</v>
       </c>
       <c r="V119" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W119" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X119" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Y119">
         <v>118</v>
       </c>
       <c r="AC119" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AF119" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AH119" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AI119" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>